<commit_message>
added poz number informatil to cutlist template  (all page)
</commit_message>
<xml_diff>
--- a/btoolsets/templatefiles/cutlist.xlsx
+++ b/btoolsets/templatefiles/cutlist.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\AdekoGit\wardatadeko\btoolsets\templatefiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ADEKO\GIT\FITZGERALDKITCHENS\btoolsets\templatefiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84704AB8-0F41-4497-8F65-32AD7554512C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{972649DB-7895-4BC6-914D-6A0AB708F05D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" tabRatio="630" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3960" yWindow="1425" windowWidth="21600" windowHeight="12645" tabRatio="630" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All Materials" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,14 @@
     <sheet name="Material 7" sheetId="15" r:id="rId8"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'All Materials'!$B$11:$M$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Material 1'!$B$11:$M$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2">'Material 2'!$B$11:$M$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3">'Material 3'!$B$11:$M$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4">'Material 4'!$B$11:$M$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5">'Material 5'!$B$11:$M$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6">'Material 6'!$B$11:$M$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7">'Material 7'!$B$11:$M$11</definedName>
     <definedName name="_FilterDatabase_0" localSheetId="0">'All Materials'!$B$11:$M$11</definedName>
     <definedName name="_FilterDatabase_0" localSheetId="1">'Material 1'!$B$11:$M$11</definedName>
     <definedName name="_FilterDatabase_0" localSheetId="2">'Material 2'!$B$11:$M$11</definedName>
@@ -39,14 +47,14 @@
     <definedName name="_FilterDatabase_0_0" localSheetId="5">'Material 5'!$B$11:$M$11</definedName>
     <definedName name="_FilterDatabase_0_0" localSheetId="6">'Material 6'!$B$11:$M$11</definedName>
     <definedName name="_FilterDatabase_0_0" localSheetId="7">'Material 7'!$B$11:$M$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'All Materials'!$B$11:$M$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Material 1'!$B$11:$M$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2">'Material 2'!$B$11:$M$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3">'Material 3'!$B$11:$M$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4">'Material 4'!$B$11:$M$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5">'Material 5'!$B$11:$M$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6">'Material 6'!$B$11:$M$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7">'Material 7'!$B$11:$M$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'All Materials'!$10:$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Material 1'!$10:$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Material 2'!$10:$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Material 3'!$10:$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Material 4'!$10:$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Material 5'!$10:$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Material 6'!$10:$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Material 7'!$10:$11</definedName>
     <definedName name="Print_Titles_0" localSheetId="0">'All Materials'!$A$10:$AKS$11</definedName>
     <definedName name="Print_Titles_0" localSheetId="1">'Material 1'!$A$10:$AKS$11</definedName>
     <definedName name="Print_Titles_0" localSheetId="2">'Material 2'!$A$10:$AKS$11</definedName>
@@ -63,21 +71,13 @@
     <definedName name="Print_Titles_0_0" localSheetId="5">'Material 5'!$A$10:$AKS$11</definedName>
     <definedName name="Print_Titles_0_0" localSheetId="6">'Material 6'!$A$10:$AKS$11</definedName>
     <definedName name="Print_Titles_0_0" localSheetId="7">'Material 7'!$A$10:$AKS$11</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'All Materials'!$10:$11</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Material 1'!$10:$11</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Material 2'!$10:$11</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Material 3'!$10:$11</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Material 4'!$10:$11</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Material 5'!$10:$11</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Material 6'!$10:$11</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Material 7'!$10:$11</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="126">
   <si>
     <t>__MATERIAL</t>
   </si>
@@ -443,6 +443,18 @@
   </si>
   <si>
     <t>Edge Band</t>
+  </si>
+  <si>
+    <t>__MODULKPOSE</t>
+  </si>
+  <si>
+    <t>__MODULKGROUPPOSE</t>
+  </si>
+  <si>
+    <t>S.POZ</t>
+  </si>
+  <si>
+    <t>POZ NO</t>
   </si>
 </sst>
 </file>
@@ -617,15 +629,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -633,27 +643,18 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -663,6 +664,9 @@
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1421,177 +1425,153 @@
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
     <col min="5" max="5" width="5.7109375" customWidth="1"/>
     <col min="6" max="13" width="6" customWidth="1"/>
-    <col min="14" max="1026" width="8.7109375"/>
+    <col min="14" max="14" width="8.7109375" customWidth="1"/>
+    <col min="15" max="1026" width="8.7109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="B1" s="16"/>
+      <c r="B1" s="17"/>
       <c r="C1" s="1" t="s">
         <v>80</v>
       </c>
       <c r="D1" s="2"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="3" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
+      <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="17"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="3" t="s">
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" t="s">
         <v>82</v>
       </c>
-      <c r="D3" s="4"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="3" t="s">
+      <c r="B4" s="13"/>
+      <c r="C4" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="3" t="s">
+      <c r="B5" s="13"/>
+      <c r="C5" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="D5" s="3"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="3" t="s">
+      <c r="B6" s="13"/>
+      <c r="C6" t="s">
         <v>85</v>
       </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
+      <c r="D6" s="3"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="5" t="s">
+      <c r="B7" s="14"/>
+      <c r="C7" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
+      <c r="D7" s="5"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="14"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="10"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="14"/>
-      <c r="Q9" s="15"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="10"/>
+      <c r="Q9" s="11"/>
     </row>
     <row r="10" spans="1:17" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
-      <c r="B10" s="20" t="s">
+      <c r="A10" s="6"/>
+      <c r="B10" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="20" t="s">
+      <c r="D10" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="E10" s="10"/>
-      <c r="F10" s="20" t="s">
+      <c r="E10" s="8"/>
+      <c r="F10" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="H10" s="20" t="s">
+      <c r="H10" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="I10" s="20"/>
-      <c r="J10" s="20"/>
-      <c r="K10" s="20"/>
-      <c r="L10" s="18" t="s">
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="L10" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="M10" s="18" t="s">
+      <c r="M10" s="12" t="s">
         <v>120</v>
       </c>
+      <c r="N10" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="O10" s="12" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="11" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="10" t="s">
+      <c r="A11" s="6"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="9" t="s">
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="I11" s="9" t="s">
+      <c r="I11" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="J11" s="9" t="s">
+      <c r="J11" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="K11" s="9" t="s">
+      <c r="K11" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="L11" s="18"/>
-      <c r="M11" s="18"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
+      <c r="N11" s="12"/>
+      <c r="O11" s="12"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
@@ -1630,10 +1610,23 @@
       <c r="M12" t="s">
         <v>10</v>
       </c>
+      <c r="N12" t="s">
+        <v>122</v>
+      </c>
+      <c r="O12" t="s">
+        <v>123</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="B11:M11" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <mergeCells count="16">
+  <mergeCells count="18">
+    <mergeCell ref="N10:N11"/>
+    <mergeCell ref="O10:O11"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
     <mergeCell ref="M10:M11"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A7:B7"/>
@@ -1645,11 +1638,6 @@
     <mergeCell ref="G10:G11"/>
     <mergeCell ref="H10:K10"/>
     <mergeCell ref="L10:L11"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.15748031496062992" bottom="0.15748031496062992" header="0.51181102362204722" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
@@ -1674,172 +1662,139 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="B1" s="16"/>
+      <c r="B1" s="17"/>
       <c r="C1" s="1" t="s">
         <v>80</v>
       </c>
       <c r="D1" s="2"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="3" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
+      <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="17"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="3" t="s">
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" t="s">
         <v>82</v>
       </c>
-      <c r="D3" s="4"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="3" t="s">
+      <c r="B4" s="13"/>
+      <c r="C4" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="3" t="s">
+      <c r="B5" s="13"/>
+      <c r="C5" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="D5" s="3"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="3" t="s">
+      <c r="B6" s="13"/>
+      <c r="C6" t="s">
         <v>85</v>
       </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
+      <c r="D6" s="3"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="5" t="s">
+      <c r="B7" s="14"/>
+      <c r="C7" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
+      <c r="D7" s="5"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="14"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="10"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="14"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="10"/>
     </row>
     <row r="10" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
-      <c r="B10" s="20" t="s">
+      <c r="A10" s="6"/>
+      <c r="B10" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="20" t="s">
+      <c r="D10" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="E10" s="11"/>
-      <c r="F10" s="20" t="s">
+      <c r="E10" s="8"/>
+      <c r="F10" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="H10" s="20" t="s">
+      <c r="H10" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="I10" s="20"/>
-      <c r="J10" s="20"/>
-      <c r="K10" s="20"/>
-      <c r="L10" s="18" t="s">
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="L10" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="M10" s="18" t="s">
+      <c r="M10" s="12" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="11" t="s">
+      <c r="A11" s="6"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="9" t="s">
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="I11" s="9" t="s">
+      <c r="I11" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="J11" s="9" t="s">
+      <c r="J11" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="K11" s="9" t="s">
+      <c r="K11" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="L11" s="18"/>
-      <c r="M11" s="18"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
@@ -1882,13 +1837,6 @@
   </sheetData>
   <autoFilter ref="B11:M11" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <mergeCells count="16">
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
     <mergeCell ref="H10:K10"/>
     <mergeCell ref="L10:L11"/>
     <mergeCell ref="M10:M11"/>
@@ -1898,6 +1846,13 @@
     <mergeCell ref="D10:D11"/>
     <mergeCell ref="F10:F11"/>
     <mergeCell ref="G10:G11"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.15748031496062992" bottom="0.15748031496062992" header="0.51181102362204722" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
@@ -1922,172 +1877,139 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="B1" s="16"/>
+      <c r="B1" s="17"/>
       <c r="C1" s="1" t="s">
         <v>80</v>
       </c>
       <c r="D1" s="2"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="3" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
+      <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="17"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="3" t="s">
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" t="s">
         <v>82</v>
       </c>
-      <c r="D3" s="4"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="3" t="s">
+      <c r="B4" s="13"/>
+      <c r="C4" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="3" t="s">
+      <c r="B5" s="13"/>
+      <c r="C5" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="D5" s="3"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="3" t="s">
+      <c r="B6" s="13"/>
+      <c r="C6" t="s">
         <v>85</v>
       </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
+      <c r="D6" s="3"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="5" t="s">
+      <c r="B7" s="14"/>
+      <c r="C7" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
+      <c r="D7" s="5"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="14"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="10"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="14"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="10"/>
     </row>
     <row r="10" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
-      <c r="B10" s="20" t="s">
+      <c r="A10" s="6"/>
+      <c r="B10" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="20" t="s">
+      <c r="D10" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="E10" s="11"/>
-      <c r="F10" s="20" t="s">
+      <c r="E10" s="8"/>
+      <c r="F10" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="H10" s="20" t="s">
+      <c r="H10" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="I10" s="20"/>
-      <c r="J10" s="20"/>
-      <c r="K10" s="20"/>
-      <c r="L10" s="18" t="s">
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="L10" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="M10" s="18" t="s">
+      <c r="M10" s="12" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="11" t="s">
+      <c r="A11" s="6"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="9" t="s">
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="I11" s="9" t="s">
+      <c r="I11" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="J11" s="9" t="s">
+      <c r="J11" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="K11" s="9" t="s">
+      <c r="K11" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="L11" s="18"/>
-      <c r="M11" s="18"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
@@ -2130,13 +2052,6 @@
   </sheetData>
   <autoFilter ref="B11:M11" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <mergeCells count="16">
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
     <mergeCell ref="H10:K10"/>
     <mergeCell ref="L10:L11"/>
     <mergeCell ref="M10:M11"/>
@@ -2146,6 +2061,13 @@
     <mergeCell ref="D10:D11"/>
     <mergeCell ref="F10:F11"/>
     <mergeCell ref="G10:G11"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.15748031496062992" bottom="0.15748031496062992" header="0.51181102362204722" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
@@ -2170,172 +2092,139 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="B1" s="16"/>
+      <c r="B1" s="17"/>
       <c r="C1" s="1" t="s">
         <v>80</v>
       </c>
       <c r="D1" s="2"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="3" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
+      <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="17"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="3" t="s">
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" t="s">
         <v>82</v>
       </c>
-      <c r="D3" s="4"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="3" t="s">
+      <c r="B4" s="13"/>
+      <c r="C4" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="3" t="s">
+      <c r="B5" s="13"/>
+      <c r="C5" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="D5" s="3"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="3" t="s">
+      <c r="B6" s="13"/>
+      <c r="C6" t="s">
         <v>85</v>
       </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
+      <c r="D6" s="3"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="5" t="s">
+      <c r="B7" s="14"/>
+      <c r="C7" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
+      <c r="D7" s="5"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="14"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="10"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="14"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="10"/>
     </row>
     <row r="10" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
-      <c r="B10" s="20" t="s">
+      <c r="A10" s="6"/>
+      <c r="B10" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="20" t="s">
+      <c r="D10" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="E10" s="11"/>
-      <c r="F10" s="20" t="s">
+      <c r="E10" s="8"/>
+      <c r="F10" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="H10" s="20" t="s">
+      <c r="H10" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="I10" s="20"/>
-      <c r="J10" s="20"/>
-      <c r="K10" s="20"/>
-      <c r="L10" s="18" t="s">
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="L10" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="M10" s="18" t="s">
+      <c r="M10" s="12" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="11" t="s">
+      <c r="A11" s="6"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="9" t="s">
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="I11" s="9" t="s">
+      <c r="I11" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="J11" s="9" t="s">
+      <c r="J11" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="K11" s="9" t="s">
+      <c r="K11" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="L11" s="18"/>
-      <c r="M11" s="18"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
@@ -2378,13 +2267,6 @@
   </sheetData>
   <autoFilter ref="B11:M11" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <mergeCells count="16">
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
     <mergeCell ref="H10:K10"/>
     <mergeCell ref="L10:L11"/>
     <mergeCell ref="M10:M11"/>
@@ -2394,6 +2276,13 @@
     <mergeCell ref="D10:D11"/>
     <mergeCell ref="F10:F11"/>
     <mergeCell ref="G10:G11"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.15748031496062992" bottom="0.15748031496062992" header="0.51181102362204722" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
@@ -2418,172 +2307,139 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="B1" s="16"/>
+      <c r="B1" s="17"/>
       <c r="C1" s="1" t="s">
         <v>80</v>
       </c>
       <c r="D1" s="2"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="3" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
+      <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="17"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="3" t="s">
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" t="s">
         <v>82</v>
       </c>
-      <c r="D3" s="4"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="3" t="s">
+      <c r="B4" s="13"/>
+      <c r="C4" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="3" t="s">
+      <c r="B5" s="13"/>
+      <c r="C5" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="D5" s="3"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="3" t="s">
+      <c r="B6" s="13"/>
+      <c r="C6" t="s">
         <v>85</v>
       </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
+      <c r="D6" s="3"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="5" t="s">
+      <c r="B7" s="14"/>
+      <c r="C7" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
+      <c r="D7" s="5"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="14"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="10"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="14"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="10"/>
     </row>
     <row r="10" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
-      <c r="B10" s="20" t="s">
+      <c r="A10" s="6"/>
+      <c r="B10" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="20" t="s">
+      <c r="D10" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="E10" s="11"/>
-      <c r="F10" s="20" t="s">
+      <c r="E10" s="8"/>
+      <c r="F10" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="H10" s="20" t="s">
+      <c r="H10" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="I10" s="20"/>
-      <c r="J10" s="20"/>
-      <c r="K10" s="20"/>
-      <c r="L10" s="18" t="s">
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="L10" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="M10" s="18" t="s">
+      <c r="M10" s="12" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="11" t="s">
+      <c r="A11" s="6"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="9" t="s">
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="I11" s="9" t="s">
+      <c r="I11" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="J11" s="9" t="s">
+      <c r="J11" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="K11" s="9" t="s">
+      <c r="K11" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="L11" s="18"/>
-      <c r="M11" s="18"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
@@ -2626,13 +2482,6 @@
   </sheetData>
   <autoFilter ref="B11:M11" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <mergeCells count="16">
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
     <mergeCell ref="H10:K10"/>
     <mergeCell ref="L10:L11"/>
     <mergeCell ref="M10:M11"/>
@@ -2642,6 +2491,13 @@
     <mergeCell ref="D10:D11"/>
     <mergeCell ref="F10:F11"/>
     <mergeCell ref="G10:G11"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.15748031496062992" bottom="0.15748031496062992" header="0.51181102362204722" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
@@ -2666,172 +2522,139 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="B1" s="16"/>
+      <c r="B1" s="17"/>
       <c r="C1" s="1" t="s">
         <v>80</v>
       </c>
       <c r="D1" s="2"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="3" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
+      <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="17"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="3" t="s">
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" t="s">
         <v>82</v>
       </c>
-      <c r="D3" s="4"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="3" t="s">
+      <c r="B4" s="13"/>
+      <c r="C4" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="3" t="s">
+      <c r="B5" s="13"/>
+      <c r="C5" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="D5" s="3"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="3" t="s">
+      <c r="B6" s="13"/>
+      <c r="C6" t="s">
         <v>85</v>
       </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
+      <c r="D6" s="3"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="5" t="s">
+      <c r="B7" s="14"/>
+      <c r="C7" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
+      <c r="D7" s="5"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="14"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="10"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="14"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="10"/>
     </row>
     <row r="10" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
-      <c r="B10" s="20" t="s">
+      <c r="A10" s="6"/>
+      <c r="B10" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="20" t="s">
+      <c r="D10" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="E10" s="11"/>
-      <c r="F10" s="20" t="s">
+      <c r="E10" s="8"/>
+      <c r="F10" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="H10" s="20" t="s">
+      <c r="H10" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="I10" s="20"/>
-      <c r="J10" s="20"/>
-      <c r="K10" s="20"/>
-      <c r="L10" s="18" t="s">
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="L10" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="M10" s="18" t="s">
+      <c r="M10" s="12" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="11" t="s">
+      <c r="A11" s="6"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="9" t="s">
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="I11" s="9" t="s">
+      <c r="I11" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="J11" s="9" t="s">
+      <c r="J11" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="K11" s="9" t="s">
+      <c r="K11" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="L11" s="18"/>
-      <c r="M11" s="18"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
@@ -2874,13 +2697,6 @@
   </sheetData>
   <autoFilter ref="B11:M11" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <mergeCells count="16">
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
     <mergeCell ref="H10:K10"/>
     <mergeCell ref="L10:L11"/>
     <mergeCell ref="M10:M11"/>
@@ -2890,6 +2706,13 @@
     <mergeCell ref="D10:D11"/>
     <mergeCell ref="F10:F11"/>
     <mergeCell ref="G10:G11"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.15748031496062992" bottom="0.15748031496062992" header="0.51181102362204722" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
@@ -2914,172 +2737,139 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="B1" s="16"/>
+      <c r="B1" s="17"/>
       <c r="C1" s="1" t="s">
         <v>80</v>
       </c>
       <c r="D1" s="2"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="3" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
+      <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="17"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="3" t="s">
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" t="s">
         <v>82</v>
       </c>
-      <c r="D3" s="4"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="3" t="s">
+      <c r="B4" s="13"/>
+      <c r="C4" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="3" t="s">
+      <c r="B5" s="13"/>
+      <c r="C5" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="D5" s="3"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="3" t="s">
+      <c r="B6" s="13"/>
+      <c r="C6" t="s">
         <v>85</v>
       </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
+      <c r="D6" s="3"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="5" t="s">
+      <c r="B7" s="14"/>
+      <c r="C7" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
+      <c r="D7" s="5"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="14"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="10"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="14"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="10"/>
     </row>
     <row r="10" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
-      <c r="B10" s="20" t="s">
+      <c r="A10" s="6"/>
+      <c r="B10" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="20" t="s">
+      <c r="D10" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="E10" s="11"/>
-      <c r="F10" s="20" t="s">
+      <c r="E10" s="8"/>
+      <c r="F10" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="H10" s="20" t="s">
+      <c r="H10" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="I10" s="20"/>
-      <c r="J10" s="20"/>
-      <c r="K10" s="20"/>
-      <c r="L10" s="18" t="s">
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="L10" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="M10" s="18" t="s">
+      <c r="M10" s="12" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="11" t="s">
+      <c r="A11" s="6"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="9" t="s">
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="I11" s="9" t="s">
+      <c r="I11" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="J11" s="9" t="s">
+      <c r="J11" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="K11" s="9" t="s">
+      <c r="K11" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="L11" s="18"/>
-      <c r="M11" s="18"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
@@ -3122,13 +2912,6 @@
   </sheetData>
   <autoFilter ref="B11:M11" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
   <mergeCells count="16">
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
     <mergeCell ref="H10:K10"/>
     <mergeCell ref="L10:L11"/>
     <mergeCell ref="M10:M11"/>
@@ -3138,6 +2921,13 @@
     <mergeCell ref="D10:D11"/>
     <mergeCell ref="F10:F11"/>
     <mergeCell ref="G10:G11"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.15748031496062992" bottom="0.15748031496062992" header="0.51181102362204722" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
@@ -3162,172 +2952,139 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="B1" s="16"/>
+      <c r="B1" s="17"/>
       <c r="C1" s="1" t="s">
         <v>80</v>
       </c>
       <c r="D1" s="2"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="3" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
+      <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="17"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="3" t="s">
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" t="s">
         <v>82</v>
       </c>
-      <c r="D3" s="4"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="3" t="s">
+      <c r="B4" s="13"/>
+      <c r="C4" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="3" t="s">
+      <c r="B5" s="13"/>
+      <c r="C5" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="D5" s="3"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="3" t="s">
+      <c r="B6" s="13"/>
+      <c r="C6" t="s">
         <v>85</v>
       </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
+      <c r="D6" s="3"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="5" t="s">
+      <c r="B7" s="14"/>
+      <c r="C7" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
+      <c r="D7" s="5"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="14"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="10"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="14"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="10"/>
     </row>
     <row r="10" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
-      <c r="B10" s="20" t="s">
+      <c r="A10" s="6"/>
+      <c r="B10" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="20" t="s">
+      <c r="D10" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="E10" s="11"/>
-      <c r="F10" s="20" t="s">
+      <c r="E10" s="8"/>
+      <c r="F10" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="H10" s="20" t="s">
+      <c r="H10" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="I10" s="20"/>
-      <c r="J10" s="20"/>
-      <c r="K10" s="20"/>
-      <c r="L10" s="18" t="s">
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="L10" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="M10" s="18" t="s">
+      <c r="M10" s="12" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="11" t="s">
+      <c r="A11" s="6"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="9" t="s">
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="I11" s="9" t="s">
+      <c r="I11" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="J11" s="9" t="s">
+      <c r="J11" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="K11" s="9" t="s">
+      <c r="K11" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="L11" s="18"/>
-      <c r="M11" s="18"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
@@ -3370,13 +3127,6 @@
   </sheetData>
   <autoFilter ref="B11:M11" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
   <mergeCells count="16">
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
     <mergeCell ref="H10:K10"/>
     <mergeCell ref="L10:L11"/>
     <mergeCell ref="M10:M11"/>
@@ -3386,6 +3136,13 @@
     <mergeCell ref="D10:D11"/>
     <mergeCell ref="F10:F11"/>
     <mergeCell ref="G10:G11"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.15748031496062992" bottom="0.15748031496062992" header="0.51181102362204722" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>

</xml_diff>